<commit_message>
Fix tower respawn map reset, event skip freezes, and add tower battle victory food bonus
</commit_message>
<xml_diff>
--- a/android/app/src/main/assets/public/files/DATA/CHR_data.xlsx
+++ b/android/app/src/main/assets/public/files/DATA/CHR_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\.antigravity\game\files\DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{583ECDD9-C5FD-41AA-BF8C-37C9821AEBDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31860DB5-D496-4B37-B86E-B1AF6A5F2A67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="420" yWindow="180" windowWidth="26205" windowHeight="14850" firstSheet="2" activeTab="13" xr2:uid="{6231C4C3-18AE-434C-A5BE-7A8D84F4A7B4}"/>
+    <workbookView xWindow="2520" yWindow="450" windowWidth="26205" windowHeight="14850" firstSheet="4" activeTab="14" xr2:uid="{6231C4C3-18AE-434C-A5BE-7A8D84F4A7B4}"/>
   </bookViews>
   <sheets>
     <sheet name="共通ﾃﾞｰﾀ" sheetId="9" r:id="rId1"/>
@@ -27,6 +27,7 @@
     <sheet name="009リフィエル" sheetId="18" r:id="rId12"/>
     <sheet name="010プロセル" sheetId="16" r:id="rId13"/>
     <sheet name="MKP" sheetId="19" r:id="rId14"/>
+    <sheet name="行動ﾊﾟﾀｰﾝ" sheetId="20" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2305" uniqueCount="603">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2343" uniqueCount="632">
   <si>
     <t>李乃果</t>
     <rPh sb="0" eb="1">
@@ -8623,22 +8624,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>戦闘中のSP減少を緩和する(10%減少)</t>
-    <rPh sb="0" eb="3">
-      <t>セントウチュウ</t>
-    </rPh>
-    <rPh sb="6" eb="8">
-      <t>ゲンショウ</t>
-    </rPh>
-    <rPh sb="9" eb="11">
-      <t>カンワ</t>
-    </rPh>
-    <rPh sb="17" eb="19">
-      <t>ゲンショウ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>MP回復時のSP減少を緩和する　MP1→HP33</t>
     <rPh sb="2" eb="4">
       <t>カイフク</t>
@@ -8665,19 +8650,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>戦闘中のSP減少を緩和する(10%減少)</t>
-    <rPh sb="0" eb="3">
-      <t>セントウチュウ</t>
-    </rPh>
-    <rPh sb="6" eb="8">
-      <t>ゲンショウ</t>
-    </rPh>
-    <rPh sb="9" eb="11">
-      <t>カンワ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>HP回復時のMP減少を10%緩和する</t>
     <rPh sb="2" eb="4">
       <t>カイフク</t>
@@ -8791,6 +8763,209 @@
     </rPh>
     <rPh sb="11" eb="13">
       <t>キロク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>戦闘中のMP減少を緩和する(10%減少)</t>
+    <rPh sb="0" eb="3">
+      <t>セントウチュウ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>ゲンショウ</t>
+    </rPh>
+    <rPh sb="9" eb="11">
+      <t>カンワ</t>
+    </rPh>
+    <rPh sb="17" eb="19">
+      <t>ゲンショウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>戦闘中のMP減少を緩和する(10%減少)</t>
+    <rPh sb="0" eb="3">
+      <t>セントウチュウ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>ゲンショウ</t>
+    </rPh>
+    <rPh sb="9" eb="11">
+      <t>カンワ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>F</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>基本的な配置は前衛</t>
+    <rPh sb="0" eb="3">
+      <t>キホンテキ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>ハイチ</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>ゼンエイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>基本的な配置は後衛</t>
+    <rPh sb="0" eb="3">
+      <t>キホンテキ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>ハイチ</t>
+    </rPh>
+    <rPh sb="7" eb="8">
+      <t>ウシ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>M</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>前後位置は隊列設定で決められた位置に従う。</t>
+    <rPh sb="0" eb="2">
+      <t>ゼンゴ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>イチ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>タイレツ</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>セッテイ</t>
+    </rPh>
+    <rPh sb="10" eb="11">
+      <t>キ</t>
+    </rPh>
+    <rPh sb="15" eb="17">
+      <t>イチ</t>
+    </rPh>
+    <rPh sb="18" eb="19">
+      <t>シタガ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>F,M,B</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>誰も前衛にいないと前衛に出る</t>
+  </si>
+  <si>
+    <t>他のメンバーが1秒以内にレーン移動していたら移動しない</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>他にメンバーがいて、全メンバーの中で最もHPが低くなると後列に下がる。</t>
+    <rPh sb="0" eb="1">
+      <t>ホカ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>F,B,M</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>前衛にいるとき自分の正面に自分の属性の防御力の高い(属性値100未満)キャラクターが来たらレーンを移動する。</t>
+    <rPh sb="0" eb="2">
+      <t>ゼンエイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>F,M</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>前列にいるとき敵の前列にいるキャラクターが自分の属性の防御力の高い(属性値100未満)キャラクターでなければその正面に移動する。</t>
+    <rPh sb="0" eb="2">
+      <t>ゼンレツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ランダムで左右どちらかのレーンを確認し、誰もいないとそちらに移動する。</t>
+  </si>
+  <si>
+    <t>M,B</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>前衛にいるとき、目の前に誰かがいたら左右どちらかのレーンへ移動する。</t>
+  </si>
+  <si>
+    <t>後列から動かない。右端か左端近いほうにレーン移動しようとする。</t>
+  </si>
+  <si>
+    <t>回復型</t>
+    <rPh sb="0" eb="3">
+      <t>カイフクガタ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>味方の2人以上がHPの5%以上を失っていれば撃つ</t>
+  </si>
+  <si>
+    <t>基本</t>
+    <rPh sb="0" eb="2">
+      <t>キホン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>※雑魚戦</t>
+  </si>
+  <si>
+    <t>雑魚敵が画面に20匹以上、敵の残り数がまだ半分より多ければ必殺技を撃つ</t>
+  </si>
+  <si>
+    <t>※魔女戦</t>
+  </si>
+  <si>
+    <t>ゲージがたまれば撃つ</t>
+  </si>
+  <si>
+    <t>6秒以内に他のメンバーが必殺技を撃っていたら撃たない。</t>
+  </si>
+  <si>
+    <t>必殺技を撃つときは1/2で前衛中央に向かって移動して撃とうとする。1/2で移動せずそのまま撃つ。</t>
+  </si>
+  <si>
+    <t>必殺技を撃つときは1/2で後衛中央に向かって移動して撃とうとする。1/2で移動せずそのまま撃つ。</t>
+    <rPh sb="13" eb="15">
+      <t>コウエイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>回復、補助</t>
+    <rPh sb="0" eb="2">
+      <t>カイフク</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>ホジョ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>必殺技を撃つときに発動場所にこだわらず、どこでも撃つ</t>
+    <rPh sb="9" eb="13">
+      <t>ハツドウバショ</t>
+    </rPh>
+    <rPh sb="24" eb="25">
+      <t>ウ</t>
     </rPh>
     <phoneticPr fontId="1"/>
   </si>
@@ -15962,7 +16137,7 @@
         <v>554</v>
       </c>
       <c r="C10" t="s">
-        <v>593</v>
+        <v>601</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.4">
@@ -15973,7 +16148,7 @@
         <v>556</v>
       </c>
       <c r="C11" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.4">
@@ -16033,7 +16208,7 @@
         <v>564</v>
       </c>
       <c r="C18" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.4">
@@ -16071,7 +16246,7 @@
         <v>583</v>
       </c>
       <c r="C23" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.4">
@@ -16120,7 +16295,7 @@
         <v>586</v>
       </c>
       <c r="C29" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.4">
@@ -16153,7 +16328,7 @@
         <v>589</v>
       </c>
       <c r="C32" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.4">
@@ -16169,22 +16344,22 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.4">
@@ -16195,6 +16370,167 @@
     <row r="41" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
         <v>592</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F7E82BA-2162-4D1A-BF6D-A9248D636709}">
+  <dimension ref="B1:D21"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <sheetData>
+    <row r="1" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B1" t="s">
+        <v>603</v>
+      </c>
+      <c r="C1" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B2" t="s">
+        <v>575</v>
+      </c>
+      <c r="C2" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B3" t="s">
+        <v>606</v>
+      </c>
+      <c r="C3" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B4" t="s">
+        <v>608</v>
+      </c>
+      <c r="C4" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B5" t="s">
+        <v>603</v>
+      </c>
+      <c r="C5" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B6" t="s">
+        <v>608</v>
+      </c>
+      <c r="C6" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B7" t="s">
+        <v>612</v>
+      </c>
+      <c r="C7" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B8" t="s">
+        <v>614</v>
+      </c>
+      <c r="C8" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B9" t="s">
+        <v>603</v>
+      </c>
+      <c r="C9" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B11" t="s">
+        <v>617</v>
+      </c>
+      <c r="C11" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B13" t="s">
+        <v>575</v>
+      </c>
+      <c r="C13" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B15" t="s">
+        <v>620</v>
+      </c>
+      <c r="C15" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B16" t="s">
+        <v>622</v>
+      </c>
+      <c r="C16" t="s">
+        <v>623</v>
+      </c>
+      <c r="D16" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B17" t="s">
+        <v>622</v>
+      </c>
+      <c r="C17" t="s">
+        <v>625</v>
+      </c>
+      <c r="D17" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B18" t="s">
+        <v>622</v>
+      </c>
+      <c r="C18" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B19" t="s">
+        <v>603</v>
+      </c>
+      <c r="C19" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B20" t="s">
+        <v>575</v>
+      </c>
+      <c r="C20" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B21" t="s">
+        <v>630</v>
+      </c>
+      <c r="C21" t="s">
+        <v>631</v>
       </c>
     </row>
   </sheetData>

</xml_diff>